<commit_message>
Incorporación de valores 2024
Se incorporan datos para el año 2024
</commit_message>
<xml_diff>
--- a/Variables.xlsx
+++ b/Variables.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\roesc\Desktop\data_final\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\roesc\Desktop\hospital-efficiency-dashboard_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70D4F38A-CE18-4B8E-BE37-1A25AB2C1644}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A154EC54-BFF7-4391-B529-676295B18342}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{80FCD92B-D29F-4CEC-AE31-37AC2274FD6E}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="588" uniqueCount="140">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="664" uniqueCount="166">
   <si>
     <t>Serie A21</t>
   </si>
@@ -458,6 +458,84 @@
   </si>
   <si>
     <t>ATENCIONES ALTA, MEDIANA Y BAJA COMPLEJIDAD</t>
+  </si>
+  <si>
+    <t>2024 (Sección E)</t>
+  </si>
+  <si>
+    <t>Cirugía General</t>
+  </si>
+  <si>
+    <t>Cirugía Cardiovascular</t>
+  </si>
+  <si>
+    <t>Cirugía Maxilofacial</t>
+  </si>
+  <si>
+    <t>Cirugía Tórax</t>
+  </si>
+  <si>
+    <t>Traumatología</t>
+  </si>
+  <si>
+    <t>Neurocirugía</t>
+  </si>
+  <si>
+    <t>Otorrinolaringología</t>
+  </si>
+  <si>
+    <t>Oftalmología</t>
+  </si>
+  <si>
+    <t>Obstetricia Y Ginecología</t>
+  </si>
+  <si>
+    <t>Ginecología</t>
+  </si>
+  <si>
+    <t>Urología</t>
+  </si>
+  <si>
+    <t>Resto Especialidades</t>
+  </si>
+  <si>
+    <t>Odontología</t>
+  </si>
+  <si>
+    <t>2024 (Sección A1,A3)</t>
+  </si>
+  <si>
+    <t>Atención Médica Niño y Adulto</t>
+  </si>
+  <si>
+    <t>Atención Médica Gineco-Obstetra</t>
+  </si>
+  <si>
+    <t>Atención por Matrona/ón</t>
+  </si>
+  <si>
+    <t>Atención por Odontólogo/a</t>
+  </si>
+  <si>
+    <t>Médico</t>
+  </si>
+  <si>
+    <t>Enfermera /o</t>
+  </si>
+  <si>
+    <t>Matrona /ón</t>
+  </si>
+  <si>
+    <t>Kinesiólogo/a</t>
+  </si>
+  <si>
+    <t>Técnico en Enfermería</t>
+  </si>
+  <si>
+    <t>Otros Profesionales</t>
+  </si>
+  <si>
+    <t>2024 (Sección I)</t>
   </si>
 </sst>
 </file>
@@ -834,7 +912,16 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -842,15 +929,6 @@
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1200,18 +1278,18 @@
       </c>
     </row>
     <row r="4" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="C4" s="31" t="s">
+      <c r="C4" s="32" t="s">
         <v>15</v>
       </c>
-      <c r="D4" s="31"/>
-      <c r="F4" s="31" t="s">
+      <c r="D4" s="32"/>
+      <c r="F4" s="32" t="s">
         <v>16</v>
       </c>
-      <c r="G4" s="31"/>
-      <c r="I4" s="31" t="s">
+      <c r="G4" s="32"/>
+      <c r="I4" s="32" t="s">
         <v>17</v>
       </c>
-      <c r="J4" s="31"/>
+      <c r="J4" s="32"/>
     </row>
     <row r="5" spans="2:10" x14ac:dyDescent="0.25">
       <c r="C5" s="2">
@@ -1470,18 +1548,18 @@
       </c>
     </row>
     <row r="20" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="C20" s="31" t="s">
+      <c r="C20" s="32" t="s">
         <v>19</v>
       </c>
-      <c r="D20" s="31"/>
-      <c r="F20" s="31" t="s">
+      <c r="D20" s="32"/>
+      <c r="F20" s="32" t="s">
         <v>20</v>
       </c>
-      <c r="G20" s="31"/>
-      <c r="I20" s="31" t="s">
+      <c r="G20" s="32"/>
+      <c r="I20" s="32" t="s">
         <v>21</v>
       </c>
-      <c r="J20" s="31"/>
+      <c r="J20" s="32"/>
     </row>
     <row r="21" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C21" s="3">
@@ -1724,18 +1802,18 @@
       </c>
     </row>
     <row r="34" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="C34" s="31" t="s">
+      <c r="C34" s="32" t="s">
         <v>22</v>
       </c>
-      <c r="D34" s="31"/>
-      <c r="F34" s="31" t="s">
+      <c r="D34" s="32"/>
+      <c r="F34" s="32" t="s">
         <v>23</v>
       </c>
-      <c r="G34" s="31"/>
-      <c r="I34" s="31" t="s">
+      <c r="G34" s="32"/>
+      <c r="I34" s="32" t="s">
         <v>24</v>
       </c>
-      <c r="J34" s="31"/>
+      <c r="J34" s="32"/>
     </row>
     <row r="35" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C35" s="3">
@@ -1978,117 +2056,199 @@
       </c>
     </row>
     <row r="48" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="F48" s="31" t="s">
+      <c r="F48" s="32" t="s">
         <v>26</v>
       </c>
-      <c r="G48" s="31"/>
-    </row>
-    <row r="49" spans="6:7" x14ac:dyDescent="0.25">
+      <c r="G48" s="32"/>
+      <c r="I48" s="32" t="s">
+        <v>140</v>
+      </c>
+      <c r="J48" s="32"/>
+    </row>
+    <row r="49" spans="6:10" x14ac:dyDescent="0.25">
       <c r="F49" s="3">
         <v>21500600</v>
       </c>
       <c r="G49" s="4" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="50" spans="6:7" x14ac:dyDescent="0.25">
+      <c r="I49" s="3">
+        <v>21500600</v>
+      </c>
+      <c r="J49" s="4" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="50" spans="6:10" x14ac:dyDescent="0.25">
       <c r="F50" s="3">
         <v>21600800</v>
       </c>
       <c r="G50" s="4" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="51" spans="6:7" x14ac:dyDescent="0.25">
+      <c r="I50" s="3">
+        <v>21600800</v>
+      </c>
+      <c r="J50" s="4" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="51" spans="6:10" x14ac:dyDescent="0.25">
       <c r="F51" s="3">
         <v>21600900</v>
       </c>
       <c r="G51" s="4" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="52" spans="6:7" x14ac:dyDescent="0.25">
+      <c r="I51" s="3">
+        <v>21600900</v>
+      </c>
+      <c r="J51" s="4" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="52" spans="6:10" x14ac:dyDescent="0.25">
       <c r="F52" s="3">
         <v>21700100</v>
       </c>
       <c r="G52" s="4" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="53" spans="6:7" x14ac:dyDescent="0.25">
+      <c r="I52" s="3">
+        <v>21700100</v>
+      </c>
+      <c r="J52" s="4" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="53" spans="6:10" x14ac:dyDescent="0.25">
       <c r="F53" s="3">
         <v>21500700</v>
       </c>
       <c r="G53" s="4" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="54" spans="6:7" x14ac:dyDescent="0.25">
+      <c r="I53" s="3">
+        <v>21500700</v>
+      </c>
+      <c r="J53" s="4" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="54" spans="6:10" x14ac:dyDescent="0.25">
       <c r="F54" s="3">
         <v>21500800</v>
       </c>
       <c r="G54" s="4" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="55" spans="6:7" x14ac:dyDescent="0.25">
+      <c r="I54" s="3">
+        <v>21500800</v>
+      </c>
+      <c r="J54" s="4" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="55" spans="6:10" x14ac:dyDescent="0.25">
       <c r="F55" s="3">
         <v>21700300</v>
       </c>
       <c r="G55" s="4" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="56" spans="6:7" x14ac:dyDescent="0.25">
+      <c r="I55" s="3">
+        <v>21700300</v>
+      </c>
+      <c r="J55" s="4" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="56" spans="6:10" x14ac:dyDescent="0.25">
       <c r="F56" s="3">
         <v>21700400</v>
       </c>
       <c r="G56" s="4" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="57" spans="6:7" x14ac:dyDescent="0.25">
+      <c r="I56" s="3">
+        <v>21700400</v>
+      </c>
+      <c r="J56" s="4" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="57" spans="6:10" x14ac:dyDescent="0.25">
       <c r="F57" s="3">
         <v>21700500</v>
       </c>
       <c r="G57" s="4" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="58" spans="6:7" x14ac:dyDescent="0.25">
+      <c r="I57" s="3">
+        <v>21700500</v>
+      </c>
+      <c r="J57" s="4" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="58" spans="6:10" x14ac:dyDescent="0.25">
       <c r="F58" s="3">
         <v>21700600</v>
       </c>
       <c r="G58" s="4" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="59" spans="6:7" x14ac:dyDescent="0.25">
+      <c r="I58" s="3">
+        <v>21700600</v>
+      </c>
+      <c r="J58" s="4" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="59" spans="6:10" x14ac:dyDescent="0.25">
       <c r="F59" s="3">
         <v>21500900</v>
       </c>
       <c r="G59" s="4" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="60" spans="6:7" x14ac:dyDescent="0.25">
+      <c r="I59" s="3">
+        <v>21500900</v>
+      </c>
+      <c r="J59" s="4" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="60" spans="6:10" x14ac:dyDescent="0.25">
       <c r="F60" s="3">
         <v>21700700</v>
       </c>
       <c r="G60" s="4" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="61" spans="6:7" x14ac:dyDescent="0.25">
+      <c r="I60" s="3">
+        <v>21700700</v>
+      </c>
+      <c r="J60" s="4" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="61" spans="6:10" x14ac:dyDescent="0.25">
       <c r="F61" s="6">
         <v>29101381</v>
       </c>
       <c r="G61" s="6" t="s">
         <v>25</v>
       </c>
+      <c r="I61" s="3">
+        <v>29101381</v>
+      </c>
+      <c r="J61" s="4" t="s">
+        <v>153</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="10">
+  <mergeCells count="11">
     <mergeCell ref="C34:D34"/>
     <mergeCell ref="F34:G34"/>
     <mergeCell ref="I34:J34"/>
@@ -2099,6 +2259,7 @@
     <mergeCell ref="C20:D20"/>
     <mergeCell ref="F20:G20"/>
     <mergeCell ref="I20:J20"/>
+    <mergeCell ref="I48:J48"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -2128,18 +2289,18 @@
       </c>
     </row>
     <row r="4" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="C4" s="31" t="s">
+      <c r="C4" s="32" t="s">
         <v>73</v>
       </c>
-      <c r="D4" s="31"/>
-      <c r="F4" s="31" t="s">
+      <c r="D4" s="32"/>
+      <c r="F4" s="32" t="s">
         <v>74</v>
       </c>
-      <c r="G4" s="31"/>
-      <c r="I4" s="31" t="s">
+      <c r="G4" s="32"/>
+      <c r="I4" s="32" t="s">
         <v>38</v>
       </c>
-      <c r="J4" s="31"/>
+      <c r="J4" s="32"/>
     </row>
     <row r="5" spans="2:10" x14ac:dyDescent="0.25">
       <c r="C5" s="23" t="s">
@@ -2342,18 +2503,18 @@
       </c>
     </row>
     <row r="16" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="C16" s="35" t="s">
+      <c r="C16" s="33" t="s">
         <v>82</v>
       </c>
-      <c r="D16" s="36"/>
-      <c r="F16" s="35" t="s">
+      <c r="D16" s="34"/>
+      <c r="F16" s="33" t="s">
         <v>83</v>
       </c>
-      <c r="G16" s="36"/>
-      <c r="I16" s="35" t="s">
+      <c r="G16" s="34"/>
+      <c r="I16" s="33" t="s">
         <v>84</v>
       </c>
-      <c r="J16" s="36"/>
+      <c r="J16" s="34"/>
     </row>
     <row r="17" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C17" s="23" t="s">
@@ -2536,18 +2697,18 @@
       </c>
     </row>
     <row r="27" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="C27" s="31" t="s">
+      <c r="C27" s="32" t="s">
         <v>85</v>
       </c>
-      <c r="D27" s="31"/>
-      <c r="F27" s="31" t="s">
+      <c r="D27" s="32"/>
+      <c r="F27" s="32" t="s">
         <v>86</v>
       </c>
-      <c r="G27" s="31"/>
-      <c r="I27" s="31" t="s">
+      <c r="G27" s="32"/>
+      <c r="I27" s="32" t="s">
         <v>87</v>
       </c>
-      <c r="J27" s="31"/>
+      <c r="J27" s="32"/>
     </row>
     <row r="28" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C28" s="23" t="s">
@@ -2744,10 +2905,14 @@
       </c>
     </row>
     <row r="39" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="F39" s="31" t="s">
+      <c r="F39" s="32" t="s">
         <v>88</v>
       </c>
-      <c r="G39" s="31"/>
+      <c r="G39" s="32"/>
+      <c r="I39" s="32" t="s">
+        <v>154</v>
+      </c>
+      <c r="J39" s="32"/>
     </row>
     <row r="40" spans="3:10" x14ac:dyDescent="0.25">
       <c r="F40" s="23" t="s">
@@ -2756,6 +2921,12 @@
       <c r="G40" s="12" t="s">
         <v>29</v>
       </c>
+      <c r="I40" s="23" t="s">
+        <v>28</v>
+      </c>
+      <c r="J40" s="12" t="s">
+        <v>155</v>
+      </c>
     </row>
     <row r="41" spans="3:10" ht="21" x14ac:dyDescent="0.25">
       <c r="F41" s="23" t="s">
@@ -2764,6 +2935,12 @@
       <c r="G41" s="13" t="s">
         <v>31</v>
       </c>
+      <c r="I41" s="23" t="s">
+        <v>30</v>
+      </c>
+      <c r="J41" s="12" t="s">
+        <v>156</v>
+      </c>
     </row>
     <row r="42" spans="3:10" x14ac:dyDescent="0.25">
       <c r="F42" s="23" t="s">
@@ -2772,6 +2949,12 @@
       <c r="G42" s="12" t="s">
         <v>41</v>
       </c>
+      <c r="I42" s="23" t="s">
+        <v>32</v>
+      </c>
+      <c r="J42" s="12" t="s">
+        <v>157</v>
+      </c>
     </row>
     <row r="43" spans="3:10" x14ac:dyDescent="0.25">
       <c r="F43" s="23" t="s">
@@ -2780,6 +2963,12 @@
       <c r="G43" s="12" t="s">
         <v>42</v>
       </c>
+      <c r="I43" s="23" t="s">
+        <v>39</v>
+      </c>
+      <c r="J43" s="12" t="s">
+        <v>158</v>
+      </c>
     </row>
     <row r="44" spans="3:10" x14ac:dyDescent="0.25">
       <c r="F44" s="23" t="s">
@@ -2788,6 +2977,12 @@
       <c r="G44" s="4" t="s">
         <v>35</v>
       </c>
+      <c r="I44" s="23" t="s">
+        <v>75</v>
+      </c>
+      <c r="J44" s="12" t="s">
+        <v>159</v>
+      </c>
     </row>
     <row r="45" spans="3:10" x14ac:dyDescent="0.25">
       <c r="F45" s="23" t="s">
@@ -2796,6 +2991,12 @@
       <c r="G45" s="4" t="s">
         <v>67</v>
       </c>
+      <c r="I45" s="23" t="s">
+        <v>76</v>
+      </c>
+      <c r="J45" s="12" t="s">
+        <v>160</v>
+      </c>
     </row>
     <row r="46" spans="3:10" x14ac:dyDescent="0.25">
       <c r="F46" s="23" t="s">
@@ -2804,6 +3005,12 @@
       <c r="G46" s="4" t="s">
         <v>37</v>
       </c>
+      <c r="I46" s="23" t="s">
+        <v>77</v>
+      </c>
+      <c r="J46" s="12" t="s">
+        <v>161</v>
+      </c>
     </row>
     <row r="47" spans="3:10" x14ac:dyDescent="0.25">
       <c r="F47" s="23" t="s">
@@ -2812,6 +3019,12 @@
       <c r="G47" s="4" t="s">
         <v>79</v>
       </c>
+      <c r="I47" s="23" t="s">
+        <v>78</v>
+      </c>
+      <c r="J47" s="12" t="s">
+        <v>162</v>
+      </c>
     </row>
     <row r="48" spans="3:10" x14ac:dyDescent="0.25">
       <c r="F48" s="23" t="s">
@@ -2820,17 +3033,29 @@
       <c r="G48" s="4" t="s">
         <v>70</v>
       </c>
-    </row>
-    <row r="49" spans="6:7" x14ac:dyDescent="0.25">
+      <c r="I48" s="23" t="s">
+        <v>80</v>
+      </c>
+      <c r="J48" s="12" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="49" spans="6:10" x14ac:dyDescent="0.25">
       <c r="F49" s="23" t="s">
         <v>81</v>
       </c>
       <c r="G49" s="4" t="s">
         <v>72</v>
       </c>
+      <c r="I49" s="23" t="s">
+        <v>81</v>
+      </c>
+      <c r="J49" s="12" t="s">
+        <v>164</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="10">
+  <mergeCells count="11">
     <mergeCell ref="C27:D27"/>
     <mergeCell ref="F27:G27"/>
     <mergeCell ref="I27:J27"/>
@@ -2841,6 +3066,7 @@
     <mergeCell ref="C16:D16"/>
     <mergeCell ref="F16:G16"/>
     <mergeCell ref="I16:J16"/>
+    <mergeCell ref="I39:J39"/>
   </mergeCells>
   <dataValidations count="5">
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Error" error="Por favor ingrese números enteros" sqref="F5:F9" xr:uid="{56DC97B0-96CD-4ECF-87DD-BC20EDC6A53E}"/>
@@ -2877,36 +3103,36 @@
     <col min="3" max="3" width="10.5703125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="44" customWidth="1"/>
     <col min="6" max="6" width="13.85546875" customWidth="1"/>
-    <col min="7" max="7" width="44.42578125" customWidth="1"/>
+    <col min="7" max="7" width="53.5703125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="41.5703125" customWidth="1"/>
+    <col min="10" max="10" width="53.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B2" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="D2" s="32" t="s">
+      <c r="D2" s="35" t="s">
         <v>138</v>
       </c>
-      <c r="E2" s="33"/>
-      <c r="F2" s="33"/>
-      <c r="G2" s="33"/>
-      <c r="H2" s="34"/>
+      <c r="E2" s="36"/>
+      <c r="F2" s="36"/>
+      <c r="G2" s="36"/>
+      <c r="H2" s="37"/>
     </row>
     <row r="4" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="C4" s="31" t="s">
+      <c r="C4" s="32" t="s">
         <v>62</v>
       </c>
-      <c r="D4" s="31"/>
-      <c r="F4" s="31" t="s">
+      <c r="D4" s="32"/>
+      <c r="F4" s="32" t="s">
         <v>63</v>
       </c>
-      <c r="G4" s="31"/>
-      <c r="I4" s="31" t="s">
+      <c r="G4" s="32"/>
+      <c r="I4" s="32" t="s">
         <v>64</v>
       </c>
-      <c r="J4" s="31"/>
+      <c r="J4" s="32"/>
     </row>
     <row r="5" spans="2:10" x14ac:dyDescent="0.25">
       <c r="C5" s="24">
@@ -3273,18 +3499,18 @@
       <c r="D23" s="28"/>
     </row>
     <row r="24" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="C24" s="35" t="s">
+      <c r="C24" s="33" t="s">
         <v>109</v>
       </c>
-      <c r="D24" s="36"/>
-      <c r="F24" s="31" t="s">
+      <c r="D24" s="34"/>
+      <c r="F24" s="32" t="s">
         <v>110</v>
       </c>
-      <c r="G24" s="31"/>
-      <c r="I24" s="31" t="s">
+      <c r="G24" s="32"/>
+      <c r="I24" s="32" t="s">
         <v>111</v>
       </c>
-      <c r="J24" s="31"/>
+      <c r="J24" s="32"/>
     </row>
     <row r="25" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C25" s="24">
@@ -3667,13 +3893,13 @@
       </c>
     </row>
     <row r="44" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="C44" s="37">
+      <c r="C44" s="31">
         <v>99100270</v>
       </c>
       <c r="D44" s="25" t="s">
         <v>107</v>
       </c>
-      <c r="F44" s="37">
+      <c r="F44" s="31">
         <v>99100270</v>
       </c>
       <c r="G44" s="25" t="s">
@@ -3701,18 +3927,18 @@
       </c>
     </row>
     <row r="47" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="C47" s="35" t="s">
+      <c r="C47" s="33" t="s">
         <v>113</v>
       </c>
-      <c r="D47" s="36"/>
-      <c r="F47" s="35" t="s">
+      <c r="D47" s="34"/>
+      <c r="F47" s="33" t="s">
         <v>112</v>
       </c>
-      <c r="G47" s="36"/>
-      <c r="I47" s="35" t="s">
+      <c r="G47" s="34"/>
+      <c r="I47" s="33" t="s">
         <v>115</v>
       </c>
-      <c r="J47" s="36"/>
+      <c r="J47" s="34"/>
     </row>
     <row r="48" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C48" s="24">
@@ -4075,13 +4301,13 @@
       </c>
     </row>
     <row r="66" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="C66" s="37">
+      <c r="C66" s="31">
         <v>99100270</v>
       </c>
       <c r="D66" s="25" t="s">
         <v>107</v>
       </c>
-      <c r="F66" s="37">
+      <c r="F66" s="31">
         <v>99100270</v>
       </c>
       <c r="G66" s="25" t="s">
@@ -4107,7 +4333,7 @@
       <c r="G67" s="26" t="s">
         <v>114</v>
       </c>
-      <c r="I67" s="37" t="s">
+      <c r="I67" s="31" t="s">
         <v>134</v>
       </c>
       <c r="J67" s="25" t="s">
@@ -4123,10 +4349,14 @@
       </c>
     </row>
     <row r="70" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="F70" s="31" t="s">
+      <c r="F70" s="32" t="s">
         <v>137</v>
       </c>
-      <c r="G70" s="31"/>
+      <c r="G70" s="32"/>
+      <c r="I70" s="32" t="s">
+        <v>165</v>
+      </c>
+      <c r="J70" s="32"/>
     </row>
     <row r="71" spans="3:10" x14ac:dyDescent="0.25">
       <c r="F71" s="24" t="s">
@@ -4135,6 +4365,12 @@
       <c r="G71" s="18" t="s">
         <v>89</v>
       </c>
+      <c r="I71" s="24" t="s">
+        <v>116</v>
+      </c>
+      <c r="J71" s="18" t="s">
+        <v>89</v>
+      </c>
     </row>
     <row r="72" spans="3:10" x14ac:dyDescent="0.25">
       <c r="F72" s="24" t="s">
@@ -4143,6 +4379,12 @@
       <c r="G72" s="18" t="s">
         <v>90</v>
       </c>
+      <c r="I72" s="24" t="s">
+        <v>117</v>
+      </c>
+      <c r="J72" s="18" t="s">
+        <v>90</v>
+      </c>
     </row>
     <row r="73" spans="3:10" x14ac:dyDescent="0.25">
       <c r="F73" s="24" t="s">
@@ -4151,6 +4393,12 @@
       <c r="G73" s="18" t="s">
         <v>91</v>
       </c>
+      <c r="I73" s="24" t="s">
+        <v>118</v>
+      </c>
+      <c r="J73" s="18" t="s">
+        <v>91</v>
+      </c>
     </row>
     <row r="74" spans="3:10" x14ac:dyDescent="0.25">
       <c r="F74" s="24" t="s">
@@ -4159,6 +4407,12 @@
       <c r="G74" s="18" t="s">
         <v>92</v>
       </c>
+      <c r="I74" s="24" t="s">
+        <v>119</v>
+      </c>
+      <c r="J74" s="18" t="s">
+        <v>92</v>
+      </c>
     </row>
     <row r="75" spans="3:10" x14ac:dyDescent="0.25">
       <c r="F75" s="24" t="s">
@@ -4167,6 +4421,12 @@
       <c r="G75" s="18" t="s">
         <v>93</v>
       </c>
+      <c r="I75" s="24" t="s">
+        <v>120</v>
+      </c>
+      <c r="J75" s="18" t="s">
+        <v>93</v>
+      </c>
     </row>
     <row r="76" spans="3:10" x14ac:dyDescent="0.25">
       <c r="F76" s="24" t="s">
@@ -4175,6 +4435,12 @@
       <c r="G76" s="18" t="s">
         <v>94</v>
       </c>
+      <c r="I76" s="24" t="s">
+        <v>121</v>
+      </c>
+      <c r="J76" s="18" t="s">
+        <v>94</v>
+      </c>
     </row>
     <row r="77" spans="3:10" x14ac:dyDescent="0.25">
       <c r="F77" s="24" t="s">
@@ -4183,6 +4449,12 @@
       <c r="G77" s="18" t="s">
         <v>95</v>
       </c>
+      <c r="I77" s="24" t="s">
+        <v>122</v>
+      </c>
+      <c r="J77" s="18" t="s">
+        <v>95</v>
+      </c>
     </row>
     <row r="78" spans="3:10" x14ac:dyDescent="0.25">
       <c r="F78" s="24" t="s">
@@ -4191,6 +4463,12 @@
       <c r="G78" s="18" t="s">
         <v>96</v>
       </c>
+      <c r="I78" s="24" t="s">
+        <v>123</v>
+      </c>
+      <c r="J78" s="18" t="s">
+        <v>96</v>
+      </c>
     </row>
     <row r="79" spans="3:10" x14ac:dyDescent="0.25">
       <c r="F79" s="24" t="s">
@@ -4199,6 +4477,12 @@
       <c r="G79" s="18" t="s">
         <v>97</v>
       </c>
+      <c r="I79" s="24" t="s">
+        <v>124</v>
+      </c>
+      <c r="J79" s="18" t="s">
+        <v>97</v>
+      </c>
     </row>
     <row r="80" spans="3:10" x14ac:dyDescent="0.25">
       <c r="F80" s="24" t="s">
@@ -4207,97 +4491,169 @@
       <c r="G80" s="18" t="s">
         <v>98</v>
       </c>
-    </row>
-    <row r="81" spans="6:7" x14ac:dyDescent="0.25">
+      <c r="I80" s="24" t="s">
+        <v>125</v>
+      </c>
+      <c r="J80" s="18" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="81" spans="6:10" x14ac:dyDescent="0.25">
       <c r="F81" s="24" t="s">
         <v>126</v>
       </c>
       <c r="G81" s="18" t="s">
         <v>99</v>
       </c>
-    </row>
-    <row r="82" spans="6:7" x14ac:dyDescent="0.25">
+      <c r="I81" s="24" t="s">
+        <v>126</v>
+      </c>
+      <c r="J81" s="18" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="82" spans="6:10" x14ac:dyDescent="0.25">
       <c r="F82" s="24" t="s">
         <v>127</v>
       </c>
       <c r="G82" s="18" t="s">
         <v>101</v>
       </c>
-    </row>
-    <row r="83" spans="6:7" x14ac:dyDescent="0.25">
+      <c r="I82" s="24" t="s">
+        <v>127</v>
+      </c>
+      <c r="J82" s="18" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="83" spans="6:10" x14ac:dyDescent="0.25">
       <c r="F83" s="24" t="s">
         <v>128</v>
       </c>
       <c r="G83" s="18" t="s">
         <v>102</v>
       </c>
-    </row>
-    <row r="84" spans="6:7" x14ac:dyDescent="0.25">
-      <c r="F84" s="24" t="s">
-        <v>129</v>
+      <c r="I83" s="24" t="s">
+        <v>128</v>
+      </c>
+      <c r="J83" s="18" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="84" spans="6:10" x14ac:dyDescent="0.25">
+      <c r="F84" s="24">
+        <v>17011003</v>
       </c>
       <c r="G84" s="18" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="85" spans="6:7" x14ac:dyDescent="0.25">
+      <c r="I84" s="24" t="s">
+        <v>129</v>
+      </c>
+      <c r="J84" s="18" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="85" spans="6:10" x14ac:dyDescent="0.25">
       <c r="F85" s="24" t="s">
         <v>130</v>
       </c>
       <c r="G85" s="18" t="s">
         <v>104</v>
       </c>
-    </row>
-    <row r="86" spans="6:7" x14ac:dyDescent="0.25">
+      <c r="I85" s="24" t="s">
+        <v>130</v>
+      </c>
+      <c r="J85" s="18" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="86" spans="6:10" x14ac:dyDescent="0.25">
       <c r="F86" s="24" t="s">
         <v>131</v>
       </c>
       <c r="G86" s="18" t="s">
         <v>105</v>
       </c>
-    </row>
-    <row r="87" spans="6:7" x14ac:dyDescent="0.25">
+      <c r="I86" s="24" t="s">
+        <v>131</v>
+      </c>
+      <c r="J86" s="18" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="87" spans="6:10" x14ac:dyDescent="0.25">
       <c r="F87" s="24" t="s">
         <v>132</v>
       </c>
       <c r="G87" s="18" t="s">
         <v>106</v>
       </c>
-    </row>
-    <row r="88" spans="6:7" x14ac:dyDescent="0.25">
+      <c r="I87" s="24" t="s">
+        <v>132</v>
+      </c>
+      <c r="J87" s="18" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="88" spans="6:10" x14ac:dyDescent="0.25">
       <c r="F88" s="24" t="s">
         <v>133</v>
       </c>
       <c r="G88" s="18" t="s">
         <v>60</v>
       </c>
-    </row>
-    <row r="89" spans="6:7" x14ac:dyDescent="0.25">
+      <c r="I88" s="24" t="s">
+        <v>133</v>
+      </c>
+      <c r="J88" s="18" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="89" spans="6:10" x14ac:dyDescent="0.25">
       <c r="F89" s="24">
         <v>17200110</v>
       </c>
       <c r="G89" s="18" t="s">
         <v>107</v>
       </c>
-    </row>
-    <row r="90" spans="6:7" x14ac:dyDescent="0.25">
+      <c r="I89" s="24">
+        <v>17200110</v>
+      </c>
+      <c r="J89" s="18" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="90" spans="6:10" x14ac:dyDescent="0.25">
       <c r="F90" s="24" t="s">
         <v>134</v>
       </c>
       <c r="G90" s="25" t="s">
         <v>136</v>
       </c>
-    </row>
-    <row r="91" spans="6:7" x14ac:dyDescent="0.25">
+      <c r="I90" s="24" t="s">
+        <v>134</v>
+      </c>
+      <c r="J90" s="25" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="91" spans="6:10" x14ac:dyDescent="0.25">
       <c r="F91" s="24" t="s">
         <v>135</v>
       </c>
       <c r="G91" s="26" t="s">
         <v>114</v>
       </c>
+      <c r="I91" s="24" t="s">
+        <v>135</v>
+      </c>
+      <c r="J91" s="26" t="s">
+        <v>114</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="11">
+  <mergeCells count="12">
     <mergeCell ref="D2:H2"/>
     <mergeCell ref="C47:D47"/>
     <mergeCell ref="F47:G47"/>
@@ -4309,13 +4665,14 @@
     <mergeCell ref="C24:D24"/>
     <mergeCell ref="F24:G24"/>
     <mergeCell ref="I24:J24"/>
+    <mergeCell ref="I70:J70"/>
   </mergeCells>
   <dataValidations count="2">
     <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Error" error="Por favor ingrese números enteros" sqref="F5:G22" xr:uid="{FB5955D1-5A43-45B5-A43E-EC7C5B0C2457}">
       <formula1>0</formula1>
       <formula2>1000000000</formula2>
     </dataValidation>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="ERROR" error="Por favor ingrese solo Números." sqref="F25:G45 I25:J44 C48:D67 F48:G67 I48:J68 G71:G91" xr:uid="{F82AE8EC-74B1-4730-A8C6-52B1635ED76A}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="ERROR" error="Por favor ingrese solo Números." sqref="F25:G45 I25:J44 C48:D67 F48:G67 I48:J68 G71:G91 J71:J89 J91" xr:uid="{F82AE8EC-74B1-4730-A8C6-52B1635ED76A}"/>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>